<commit_message>
polished streamlit UI - professional clinical design with CAP alerts and color coded metrics
</commit_message>
<xml_diff>
--- a/data/output-data/unmatched_cases.xlsx
+++ b/data/output-data/unmatched_cases.xlsx
@@ -492,20 +492,20 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PT00001</t>
+          <t>PT00014</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CYT-24592</t>
+          <t>CYT-42325</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>45581</v>
+        <v>45069</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ATYPICAL GLANDULAR CELLS (AGC), NOT OTHERWISE SPECIFIED</t>
+          <t>OTHER (EMC45)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -515,22 +515,22 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>LBC</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Dr. Jones</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>OTHER (EMC45)</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -545,20 +545,20 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PT00008</t>
+          <t>PT00022</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CYT-19116</t>
+          <t>CYT-73699</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>45648</v>
+        <v>45014</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>ATYPICAL SQUAMOUS CELLS, CANNOT EXCLUDE HSIL (ASC-H)</t>
+          <t>Adenocarcinoma in situ</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -568,22 +568,22 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Conventional</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Dr. Smith</t>
+          <t>Dr. Lee</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Clinic A</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>ASC-H</t>
+          <t>AIS</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -598,20 +598,20 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PT00017</t>
+          <t>PT00037</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CYT-71348</t>
+          <t>CYT-79615</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>45537</v>
+        <v>45441</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ATYPICAL SQUAMOUS CELLS OF UNDETERMINED SIGNIFICANCE (ASC-US)</t>
+          <t>Neg</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -621,22 +621,22 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Smith</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Clinic A</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>ASC-US</t>
+          <t>NILM</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -651,35 +651,35 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PT00037</t>
+          <t>PT00041</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CYT-96752</t>
+          <t>CYT-11220</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>45496</v>
+        <v>45001</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>lsil</t>
+          <t>Endometrial cells</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation</t>
+          <t>Satisfactory</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Dr. Patel</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>LSIL</t>
+          <t>AGC-EMC</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -704,35 +704,35 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PT00041</t>
+          <t>PT00049</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CYT-85880</t>
+          <t>CYT-50404</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>45179</v>
+        <v>44969</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation. Negative for intraepithelial lesion or malignancy (NILM).</t>
+          <t>NILLM</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>LBC</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Jones</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -757,45 +757,45 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PT00055</t>
+          <t>PT00056</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CYT-53540</t>
+          <t>CYT-51114</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>45110</v>
+        <v>45280</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>AGC-NEO. Endocervical adenocarcinoma in situ cannot be excluded.</t>
+          <t>Carcinoma</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation</t>
+          <t>Satisfactory</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Conventional</t>
+          <t>LBC</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Dr. Jones</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Clinic A</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>AGC-NEO</t>
+          <t>MALIGNANT</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -810,45 +810,45 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PT00063</t>
+          <t>PT00062</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CYT-97410</t>
+          <t>CYT-38010</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>45243</v>
+        <v>45618</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Atypical squamous cells, undetermined significance. Reflex HPV testing recommended.</t>
+          <t>MALIGNANT</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Adequate</t>
+          <t>Satisfactory for evaluation</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Conventional</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Patel</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Clinic A</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>MALIGNANT</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -863,45 +863,45 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PT00067</t>
+          <t>PT00064</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CYT-97012</t>
+          <t>CYT-29313</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>45454</v>
+        <v>45130</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>HSIL - SEE COMMENT. Correlate with clinical findings.</t>
+          <t>NILLM</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Satisfactory for evaluation</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>LBC</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Dr. Jones</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Clinic A</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>HSIL</t>
+          <t>NILM</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -916,20 +916,20 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PT00071</t>
+          <t>PT00065</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CYT-77889</t>
+          <t>CYT-64321</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>45107</v>
+        <v>45393</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation. Negative for intraepithelial lesion or malignancy (NILM).</t>
+          <t>Endometrial cells</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -939,7 +939,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>LBC</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -949,12 +949,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>NILM</t>
+          <t>AGC-EMC</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -969,25 +969,25 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PT00078</t>
+          <t>PT00068</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CYT-86556</t>
+          <t>CYT-97500</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>45325</v>
+        <v>45402</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>NEGATIVE FOR INTRAEPITHELIAL LESION OR MALIGNANCY</t>
+          <t>OTHER (EMC45)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Adequate</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -997,17 +997,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Dr. Smith</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Clinic A</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>NILM</t>
+          <t>OTHER (EMC45)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1022,45 +1022,45 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PT00085</t>
+          <t>PT00090</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CYT-95426</t>
+          <t>CYT-84691</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>44997</v>
+        <v>45402</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Atypical glandular cells, favor neoplasia. Further evaluation recommended.</t>
+          <t>ASC H</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Dr. Jones</t>
+          <t>Dr. Lee</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>AGC-NEO</t>
+          <t>ASC-H</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1075,20 +1075,20 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PT00089</t>
+          <t>PT00101</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CYT-92213</t>
+          <t>CYT-71524</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>45533</v>
+        <v>45218</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Negative. No significant atypia identified.</t>
+          <t>AGC-NEO</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1098,22 +1098,22 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Smith</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>NILM</t>
+          <t>AGC-NEO</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1128,25 +1128,25 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PT00090</t>
+          <t>PT00102</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CYT-79827</t>
+          <t>CYT-24953</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>45282</v>
+        <v>45416</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>ATYPICAL SQUAMOUS CELLS, CANNOT EXCLUDE HSIL (ASC-H)</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Adequate</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>ASC-H</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1181,30 +1181,30 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PT00100</t>
+          <t>PT00109</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CYT-58368</t>
+          <t>CYT-87304</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>45522</v>
+        <v>45567</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>HSIL. Features consistent with CIN 2-3. Colposcopy recommended.</t>
+          <t>LSIL</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Adequate</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>LBC</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1214,12 +1214,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>HSIL</t>
+          <t>LSIL</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1234,25 +1234,25 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PT00125</t>
+          <t>PT00118</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CYT-17104</t>
+          <t>CYT-52372</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>45350</v>
+        <v>45185</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>HIGH GRADE SQUAMOUS INTRAEPITHELIAL LESION (HSIL)</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Satisfactory</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>HSIL</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1287,25 +1287,25 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PT00127</t>
+          <t>PT00122</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CYT-92578</t>
+          <t>CYT-39451</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>44956</v>
+        <v>45022</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>AGC-NEO. Endocervical adenocarcinoma in situ cannot be excluded.</t>
+          <t>Atypical glandular cells favor neoplasia</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation</t>
+          <t>Satisfactory</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Dr. Patel</t>
+          <t>Dr. Lee</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1340,20 +1340,20 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PT00142</t>
+          <t>PT00129</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CYT-13794</t>
+          <t>CYT-95461</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>45233</v>
+        <v>45606</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Atypical squamous cells, undetermined significance. Reflex HPV testing recommended.</t>
+          <t>Malignant cells present</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1363,22 +1363,22 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Conventional</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Dr. Patel</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Clinic A</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>MALIGNANT</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1393,35 +1393,35 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PT00144</t>
+          <t>PT00134</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CYT-89887</t>
+          <t>CYT-93066</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>45007</v>
+        <v>45027</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>HSIL - SEE COMMENT. Correlate with clinical findings.</t>
+          <t>Negative cytology</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation</t>
+          <t>Adequate</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>LBC</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Patel</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>HSIL</t>
+          <t>NILM</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1446,25 +1446,25 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PT00145</t>
+          <t>PT00139</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CYT-70443</t>
+          <t>CYT-30706</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>45164</v>
+        <v>45486</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>ATYPICAL SQUAMOUS CELLS OF UNDETERMINED SIGNIFICANCE (ASC-US)</t>
+          <t>AGC-NEO</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Adequate</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1474,17 +1474,17 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Dr. Smith</t>
+          <t>Dr. Lee</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Clinic A</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>ASC-US</t>
+          <t>AGC-NEO</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1499,30 +1499,30 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PT00150</t>
+          <t>PT00145</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CYT-16428</t>
+          <t>CYT-52823</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>45629</v>
+        <v>45229</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>ATYPICAL GLANDULAR CELLS (AGC), NOT OTHERWISE SPECIFIED</t>
+          <t>Atypical glandular cells</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Adequate</t>
+          <t>Satisfactory for evaluation</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Conventional</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">

</xml_diff>

<commit_message>
streamlit UI polished - session state fix - file validation - eval mode working
</commit_message>
<xml_diff>
--- a/data/output-data/unmatched_cases.xlsx
+++ b/data/output-data/unmatched_cases.xlsx
@@ -492,20 +492,20 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PT00014</t>
+          <t>PT00001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CYT-42325</t>
+          <t>CYT-24592</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>45069</v>
+        <v>45581</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>OTHER (EMC45)</t>
+          <t>ATYPICAL GLANDULAR CELLS (AGC), NOT OTHERWISE SPECIFIED</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -515,22 +515,22 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>LBC</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Jones</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>OTHER (EMC45)</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -545,20 +545,20 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PT00022</t>
+          <t>PT00008</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CYT-73699</t>
+          <t>CYT-19116</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>45014</v>
+        <v>45648</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Adenocarcinoma in situ</t>
+          <t>ATYPICAL SQUAMOUS CELLS, CANNOT EXCLUDE HSIL (ASC-H)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -568,22 +568,22 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>Conventional</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Dr. Lee</t>
+          <t>Dr. Smith</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Clinic A</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>AIS</t>
+          <t>ASC-H</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -598,20 +598,20 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PT00037</t>
+          <t>PT00017</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CYT-79615</t>
+          <t>CYT-71348</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>45441</v>
+        <v>45537</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Neg</t>
+          <t>ATYPICAL SQUAMOUS CELLS OF UNDETERMINED SIGNIFICANCE (ASC-US)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -621,22 +621,22 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Dr. Smith</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Clinic A</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>NILM</t>
+          <t>ASC-US</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -651,35 +651,35 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PT00041</t>
+          <t>PT00037</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CYT-11220</t>
+          <t>CYT-96752</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>45001</v>
+        <v>45496</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Endometrial cells</t>
+          <t>lsil</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactory for evaluation</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Patel</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>AGC-EMC</t>
+          <t>LSIL</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -704,35 +704,35 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PT00049</t>
+          <t>PT00041</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CYT-50404</t>
+          <t>CYT-85880</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>44969</v>
+        <v>45179</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>NILLM</t>
+          <t>Satisfactory for evaluation. Negative for intraepithelial lesion or malignancy (NILM).</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Satisfactory</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>LBC</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Dr. Jones</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -757,45 +757,45 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PT00056</t>
+          <t>PT00055</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CYT-51114</t>
+          <t>CYT-53540</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>45280</v>
+        <v>45110</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Carcinoma</t>
+          <t>AGC-NEO. Endocervical adenocarcinoma in situ cannot be excluded.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactory for evaluation</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>LBC</t>
+          <t>Conventional</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Jones</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Clinic A</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>MALIGNANT</t>
+          <t>AGC-NEO</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -810,45 +810,45 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PT00062</t>
+          <t>PT00063</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CYT-38010</t>
+          <t>CYT-97410</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>45618</v>
+        <v>45243</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MALIGNANT</t>
+          <t>Atypical squamous cells, undetermined significance. Reflex HPV testing recommended.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation</t>
+          <t>Adequate</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>Conventional</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Dr. Patel</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Clinic A</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>MALIGNANT</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -863,45 +863,45 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PT00064</t>
+          <t>PT00067</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CYT-29313</t>
+          <t>CYT-97012</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>45130</v>
+        <v>45454</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>NILLM</t>
+          <t>HSIL - SEE COMMENT. Correlate with clinical findings.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>LBC</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Jones</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Clinic A</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>NILM</t>
+          <t>HSIL</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -916,20 +916,20 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PT00065</t>
+          <t>PT00071</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CYT-64321</t>
+          <t>CYT-77889</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>45393</v>
+        <v>45107</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Endometrial cells</t>
+          <t>Satisfactory for evaluation. Negative for intraepithelial lesion or malignancy (NILM).</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -939,7 +939,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>LBC</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -949,12 +949,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>AGC-EMC</t>
+          <t>NILM</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -969,25 +969,25 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PT00068</t>
+          <t>PT00078</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CYT-97500</t>
+          <t>CYT-86556</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>45402</v>
+        <v>45325</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>OTHER (EMC45)</t>
+          <t>NEGATIVE FOR INTRAEPITHELIAL LESION OR MALIGNANCY</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Adequate</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -997,17 +997,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Smith</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Clinic A</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>OTHER (EMC45)</t>
+          <t>NILM</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1022,45 +1022,45 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PT00090</t>
+          <t>PT00085</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CYT-84691</t>
+          <t>CYT-95426</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>45402</v>
+        <v>44997</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ASC H</t>
+          <t>Atypical glandular cells, favor neoplasia. Further evaluation recommended.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Satisfactory</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Dr. Lee</t>
+          <t>Dr. Jones</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>ASC-H</t>
+          <t>AGC-NEO</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1075,20 +1075,20 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PT00101</t>
+          <t>PT00089</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CYT-71524</t>
+          <t>CYT-92213</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>45218</v>
+        <v>45533</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>AGC-NEO</t>
+          <t>Negative. No significant atypia identified.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1098,22 +1098,22 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Dr. Smith</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>AGC-NEO</t>
+          <t>NILM</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1128,25 +1128,25 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PT00102</t>
+          <t>PT00090</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CYT-24953</t>
+          <t>CYT-79827</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>45416</v>
+        <v>45282</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>ATYPICAL SQUAMOUS CELLS, CANNOT EXCLUDE HSIL (ASC-H)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Adequate</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>ASC-H</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1181,30 +1181,30 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PT00109</t>
+          <t>PT00100</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CYT-87304</t>
+          <t>CYT-58368</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>45567</v>
+        <v>45522</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>LSIL</t>
+          <t>HSIL. Features consistent with CIN 2-3. Colposcopy recommended.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Adequate</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>LBC</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1214,12 +1214,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>LSIL</t>
+          <t>HSIL</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1234,25 +1234,25 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PT00118</t>
+          <t>PT00125</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CYT-52372</t>
+          <t>CYT-17104</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>45185</v>
+        <v>45350</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>HIGH GRADE SQUAMOUS INTRAEPITHELIAL LESION (HSIL)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>HSIL</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1287,25 +1287,25 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PT00122</t>
+          <t>PT00127</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CYT-39451</t>
+          <t>CYT-92578</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>45022</v>
+        <v>44956</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Atypical glandular cells favor neoplasia</t>
+          <t>AGC-NEO. Endocervical adenocarcinoma in situ cannot be excluded.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactory for evaluation</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Dr. Lee</t>
+          <t>Dr. Patel</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1340,20 +1340,20 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PT00129</t>
+          <t>PT00142</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CYT-95461</t>
+          <t>CYT-13794</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>45606</v>
+        <v>45233</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Malignant cells present</t>
+          <t>Atypical squamous cells, undetermined significance. Reflex HPV testing recommended.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1363,22 +1363,22 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>Conventional</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Patel</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Clinic A</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>MALIGNANT</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1393,35 +1393,35 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PT00134</t>
+          <t>PT00144</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CYT-93066</t>
+          <t>CYT-89887</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>45027</v>
+        <v>45007</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Negative cytology</t>
+          <t>HSIL - SEE COMMENT. Correlate with clinical findings.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Adequate</t>
+          <t>Satisfactory for evaluation</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>LBC</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Dr. Patel</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>NILM</t>
+          <t>HSIL</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1446,25 +1446,25 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PT00139</t>
+          <t>PT00145</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CYT-30706</t>
+          <t>CYT-70443</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>45486</v>
+        <v>45164</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>AGC-NEO</t>
+          <t>ATYPICAL SQUAMOUS CELLS OF UNDETERMINED SIGNIFICANCE (ASC-US)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Adequate</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1474,17 +1474,17 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Dr. Lee</t>
+          <t>Dr. Smith</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Clinic A</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>AGC-NEO</t>
+          <t>ASC-US</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1499,30 +1499,30 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PT00145</t>
+          <t>PT00150</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CYT-52823</t>
+          <t>CYT-16428</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>45229</v>
+        <v>45629</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Atypical glandular cells</t>
+          <t>ATYPICAL GLANDULAR CELLS (AGC), NOT OTHERWISE SPECIFIED</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation</t>
+          <t>Adequate</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>Conventional</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">

</xml_diff>

<commit_message>
modern visualizations - Birdsong metrics in UI and PDF - intergrade follow-up table - updated metrics.py
</commit_message>
<xml_diff>
--- a/data/output-data/unmatched_cases.xlsx
+++ b/data/output-data/unmatched_cases.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -485,6 +485,11 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>Cyto_LLM_Reasoning</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Cyto_Valid</t>
         </is>
       </c>
@@ -492,20 +497,20 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PT00001</t>
+          <t>PT00014</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CYT-24592</t>
+          <t>CYT-42325</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>45581</v>
+        <v>45069</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ATYPICAL GLANDULAR CELLS (AGC), NOT OTHERWISE SPECIFIED</t>
+          <t>OTHER (EMC45)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -515,22 +520,22 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>LBC</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Dr. Jones</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>OTHER (EMC45)</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -538,27 +543,28 @@
           <t>high</t>
         </is>
       </c>
-      <c r="K2" t="b">
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PT00008</t>
+          <t>PT00022</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CYT-19116</t>
+          <t>CYT-73699</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>45648</v>
+        <v>45014</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>ATYPICAL SQUAMOUS CELLS, CANNOT EXCLUDE HSIL (ASC-H)</t>
+          <t>Adenocarcinoma in situ</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -568,22 +574,22 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Conventional</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Dr. Smith</t>
+          <t>Dr. Lee</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Clinic A</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>ASC-H</t>
+          <t>AIS</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -591,27 +597,28 @@
           <t>high</t>
         </is>
       </c>
-      <c r="K3" t="b">
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PT00017</t>
+          <t>PT00037</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CYT-71348</t>
+          <t>CYT-79615</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>45537</v>
+        <v>45441</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ATYPICAL SQUAMOUS CELLS OF UNDETERMINED SIGNIFICANCE (ASC-US)</t>
+          <t>Neg</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -621,22 +628,22 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Smith</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Clinic A</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>ASC-US</t>
+          <t>NILM</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -644,42 +651,43 @@
           <t>high</t>
         </is>
       </c>
-      <c r="K4" t="b">
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PT00037</t>
+          <t>PT00041</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CYT-96752</t>
+          <t>CYT-11220</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>45496</v>
+        <v>45001</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>lsil</t>
+          <t>Endometrial cells</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation</t>
+          <t>Satisfactory</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Dr. Patel</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -689,7 +697,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>LSIL</t>
+          <t>AGC-EMC</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -697,42 +705,43 @@
           <t>high</t>
         </is>
       </c>
-      <c r="K5" t="b">
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PT00041</t>
+          <t>PT00049</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CYT-85880</t>
+          <t>CYT-50404</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>45179</v>
+        <v>44969</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation. Negative for intraepithelial lesion or malignancy (NILM).</t>
+          <t>NILLM</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>LBC</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Jones</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -750,52 +759,53 @@
           <t>high</t>
         </is>
       </c>
-      <c r="K6" t="b">
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PT00055</t>
+          <t>PT00056</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CYT-53540</t>
+          <t>CYT-51114</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>45110</v>
+        <v>45280</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>AGC-NEO. Endocervical adenocarcinoma in situ cannot be excluded.</t>
+          <t>Carcinoma</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation</t>
+          <t>Satisfactory</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Conventional</t>
+          <t>LBC</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Dr. Jones</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Clinic A</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>AGC-NEO</t>
+          <t>MALIGNANT</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -803,52 +813,53 @@
           <t>high</t>
         </is>
       </c>
-      <c r="K7" t="b">
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PT00063</t>
+          <t>PT00062</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CYT-97410</t>
+          <t>CYT-38010</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>45243</v>
+        <v>45618</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Atypical squamous cells, undetermined significance. Reflex HPV testing recommended.</t>
+          <t>MALIGNANT</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Adequate</t>
+          <t>Satisfactory for evaluation</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Conventional</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Patel</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Clinic A</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>MALIGNANT</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -856,52 +867,53 @@
           <t>high</t>
         </is>
       </c>
-      <c r="K8" t="b">
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PT00067</t>
+          <t>PT00064</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CYT-97012</t>
+          <t>CYT-29313</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>45454</v>
+        <v>45130</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>HSIL - SEE COMMENT. Correlate with clinical findings.</t>
+          <t>NILLM</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Satisfactory for evaluation</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>LBC</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Dr. Jones</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Clinic A</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>HSIL</t>
+          <t>NILM</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -909,27 +921,28 @@
           <t>high</t>
         </is>
       </c>
-      <c r="K9" t="b">
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PT00071</t>
+          <t>PT00065</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CYT-77889</t>
+          <t>CYT-64321</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>45107</v>
+        <v>45393</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation. Negative for intraepithelial lesion or malignancy (NILM).</t>
+          <t>Endometrial cells</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -939,7 +952,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>LBC</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -949,12 +962,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>NILM</t>
+          <t>AGC-EMC</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -962,32 +975,33 @@
           <t>high</t>
         </is>
       </c>
-      <c r="K10" t="b">
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PT00078</t>
+          <t>PT00068</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CYT-86556</t>
+          <t>CYT-97500</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>45325</v>
+        <v>45402</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>NEGATIVE FOR INTRAEPITHELIAL LESION OR MALIGNANCY</t>
+          <t>OTHER (EMC45)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Adequate</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -997,17 +1011,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Dr. Smith</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Clinic A</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>NILM</t>
+          <t>OTHER (EMC45)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1015,52 +1029,53 @@
           <t>high</t>
         </is>
       </c>
-      <c r="K11" t="b">
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PT00085</t>
+          <t>PT00090</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CYT-95426</t>
+          <t>CYT-84691</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>44997</v>
+        <v>45402</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Atypical glandular cells, favor neoplasia. Further evaluation recommended.</t>
+          <t>ASC H</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Dr. Jones</t>
+          <t>Dr. Lee</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>AGC-NEO</t>
+          <t>ASC-H</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1068,27 +1083,28 @@
           <t>high</t>
         </is>
       </c>
-      <c r="K12" t="b">
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PT00089</t>
+          <t>PT00101</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CYT-92213</t>
+          <t>CYT-71524</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>45533</v>
+        <v>45218</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Negative. No significant atypia identified.</t>
+          <t>AGC-NEO</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1098,22 +1114,22 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Smith</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>NILM</t>
+          <t>AGC-NEO</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1121,32 +1137,33 @@
           <t>high</t>
         </is>
       </c>
-      <c r="K13" t="b">
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PT00090</t>
+          <t>PT00102</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CYT-79827</t>
+          <t>CYT-24953</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>45282</v>
+        <v>45416</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>ATYPICAL SQUAMOUS CELLS, CANNOT EXCLUDE HSIL (ASC-H)</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Adequate</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1166,7 +1183,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>ASC-H</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1174,37 +1191,38 @@
           <t>high</t>
         </is>
       </c>
-      <c r="K14" t="b">
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PT00100</t>
+          <t>PT00109</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CYT-58368</t>
+          <t>CYT-87304</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>45522</v>
+        <v>45567</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>HSIL. Features consistent with CIN 2-3. Colposcopy recommended.</t>
+          <t>LSIL</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Adequate</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>LBC</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1214,12 +1232,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>HSIL</t>
+          <t>LSIL</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1227,32 +1245,33 @@
           <t>high</t>
         </is>
       </c>
-      <c r="K15" t="b">
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PT00125</t>
+          <t>PT00118</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CYT-17104</t>
+          <t>CYT-52372</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>45350</v>
+        <v>45185</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>HIGH GRADE SQUAMOUS INTRAEPITHELIAL LESION (HSIL)</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Satisfactory</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1272,7 +1291,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>HSIL</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1280,32 +1299,33 @@
           <t>high</t>
         </is>
       </c>
-      <c r="K16" t="b">
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PT00127</t>
+          <t>PT00122</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CYT-92578</t>
+          <t>CYT-39451</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>44956</v>
+        <v>45022</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>AGC-NEO. Endocervical adenocarcinoma in situ cannot be excluded.</t>
+          <t>Atypical glandular cells favor neoplasia</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation</t>
+          <t>Satisfactory</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1315,7 +1335,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Dr. Patel</t>
+          <t>Dr. Lee</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1333,27 +1353,28 @@
           <t>high</t>
         </is>
       </c>
-      <c r="K17" t="b">
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PT00142</t>
+          <t>PT00129</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CYT-13794</t>
+          <t>CYT-95461</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>45233</v>
+        <v>45606</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Atypical squamous cells, undetermined significance. Reflex HPV testing recommended.</t>
+          <t>Malignant cells present</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1363,22 +1384,22 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Conventional</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Dr. Patel</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Clinic A</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>MALIGNANT</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1386,42 +1407,43 @@
           <t>high</t>
         </is>
       </c>
-      <c r="K18" t="b">
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PT00144</t>
+          <t>PT00134</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CYT-89887</t>
+          <t>CYT-93066</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>45007</v>
+        <v>45027</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>HSIL - SEE COMMENT. Correlate with clinical findings.</t>
+          <t>Negative cytology</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation</t>
+          <t>Adequate</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>LBC</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Patel</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1431,7 +1453,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>HSIL</t>
+          <t>NILM</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1439,32 +1461,33 @@
           <t>high</t>
         </is>
       </c>
-      <c r="K19" t="b">
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PT00145</t>
+          <t>PT00139</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CYT-70443</t>
+          <t>CYT-30706</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>45164</v>
+        <v>45486</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>ATYPICAL SQUAMOUS CELLS OF UNDETERMINED SIGNIFICANCE (ASC-US)</t>
+          <t>AGC-NEO</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Adequate</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1474,17 +1497,17 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Dr. Smith</t>
+          <t>Dr. Lee</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Clinic A</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>ASC-US</t>
+          <t>AGC-NEO</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1492,37 +1515,38 @@
           <t>high</t>
         </is>
       </c>
-      <c r="K20" t="b">
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PT00150</t>
+          <t>PT00145</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CYT-16428</t>
+          <t>CYT-52823</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>45629</v>
+        <v>45229</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>ATYPICAL GLANDULAR CELLS (AGC), NOT OTHERWISE SPECIFIED</t>
+          <t>Atypical glandular cells</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Adequate</t>
+          <t>Satisfactory for evaluation</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Conventional</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1545,7 +1569,8 @@
           <t>high</t>
         </is>
       </c>
-      <c r="K21" t="b">
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
clean streamlit UI - remove duplicate results - Birdsong metrics complete
</commit_message>
<xml_diff>
--- a/data/output-data/unmatched_cases.xlsx
+++ b/data/output-data/unmatched_cases.xlsx
@@ -497,20 +497,20 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PT00014</t>
+          <t>PT00001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CYT-42325</t>
+          <t>CYT-24592</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>45069</v>
+        <v>45581</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>OTHER (EMC45)</t>
+          <t>ATYPICAL GLANDULAR CELLS (AGC), NOT OTHERWISE SPECIFIED</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -520,22 +520,22 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>LBC</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Jones</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>OTHER (EMC45)</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -551,20 +551,20 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PT00022</t>
+          <t>PT00008</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CYT-73699</t>
+          <t>CYT-19116</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>45014</v>
+        <v>45648</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Adenocarcinoma in situ</t>
+          <t>ATYPICAL SQUAMOUS CELLS, CANNOT EXCLUDE HSIL (ASC-H)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -574,22 +574,22 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>Conventional</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Dr. Lee</t>
+          <t>Dr. Smith</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Clinic A</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>AIS</t>
+          <t>ASC-H</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -605,20 +605,20 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PT00037</t>
+          <t>PT00017</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CYT-79615</t>
+          <t>CYT-71348</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>45441</v>
+        <v>45537</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Neg</t>
+          <t>ATYPICAL SQUAMOUS CELLS OF UNDETERMINED SIGNIFICANCE (ASC-US)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -628,22 +628,22 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Dr. Smith</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Clinic A</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>NILM</t>
+          <t>ASC-US</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -659,35 +659,35 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PT00041</t>
+          <t>PT00037</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CYT-11220</t>
+          <t>CYT-96752</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>45001</v>
+        <v>45496</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Endometrial cells</t>
+          <t>lsil</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactory for evaluation</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Patel</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>AGC-EMC</t>
+          <t>LSIL</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -713,35 +713,35 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PT00049</t>
+          <t>PT00041</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CYT-50404</t>
+          <t>CYT-85880</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>44969</v>
+        <v>45179</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>NILLM</t>
+          <t>Satisfactory for evaluation. Negative for intraepithelial lesion or malignancy (NILM).</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Satisfactory</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>LBC</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Dr. Jones</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -767,45 +767,45 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PT00056</t>
+          <t>PT00055</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CYT-51114</t>
+          <t>CYT-53540</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>45280</v>
+        <v>45110</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Carcinoma</t>
+          <t>AGC-NEO. Endocervical adenocarcinoma in situ cannot be excluded.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactory for evaluation</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>LBC</t>
+          <t>Conventional</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Jones</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Clinic A</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>MALIGNANT</t>
+          <t>AGC-NEO</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -821,99 +821,95 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PT00062</t>
+          <t>PT00063</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CYT-38010</t>
+          <t>CYT-97410</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>45618</v>
+        <v>45243</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MALIGNANT</t>
+          <t>Atypical squamous cells, undetermined significance. Reflex HPV testing recommended.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation</t>
+          <t>Adequate</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>Conventional</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Dr. Patel</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Clinic A</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>MALIGNANT</t>
-        </is>
-      </c>
+          <t>Main Lab</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PT00064</t>
+          <t>PT00067</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CYT-29313</t>
+          <t>CYT-97012</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>45130</v>
+        <v>45454</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>NILLM</t>
+          <t>HSIL - SEE COMMENT. Correlate with clinical findings.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>LBC</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Jones</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Clinic A</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>NILM</t>
+          <t>HSIL</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -929,20 +925,20 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PT00065</t>
+          <t>PT00071</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CYT-64321</t>
+          <t>CYT-77889</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>45393</v>
+        <v>45107</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Endometrial cells</t>
+          <t>Satisfactory for evaluation. Negative for intraepithelial lesion or malignancy (NILM).</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -952,7 +948,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>LBC</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -962,12 +958,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>AGC-EMC</t>
+          <t>NILM</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -983,25 +979,25 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PT00068</t>
+          <t>PT00078</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CYT-97500</t>
+          <t>CYT-86556</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>45402</v>
+        <v>45325</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>OTHER (EMC45)</t>
+          <t>NEGATIVE FOR INTRAEPITHELIAL LESION OR MALIGNANCY</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Adequate</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1011,17 +1007,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Smith</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Clinic A</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>OTHER (EMC45)</t>
+          <t>NILM</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1037,45 +1033,45 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PT00090</t>
+          <t>PT00085</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CYT-84691</t>
+          <t>CYT-95426</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>45402</v>
+        <v>44997</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ASC H</t>
+          <t>Atypical glandular cells, favor neoplasia. Further evaluation recommended.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Satisfactory</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Dr. Lee</t>
+          <t>Dr. Jones</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>ASC-H</t>
+          <t>AGC-NEO</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1091,20 +1087,20 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PT00101</t>
+          <t>PT00089</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CYT-71524</t>
+          <t>CYT-92213</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>45218</v>
+        <v>45533</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>AGC-NEO</t>
+          <t>Negative. No significant atypia identified.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1114,22 +1110,22 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Dr. Smith</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>AGC-NEO</t>
+          <t>NILM</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1145,25 +1141,25 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PT00102</t>
+          <t>PT00090</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CYT-24953</t>
+          <t>CYT-79827</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>45416</v>
+        <v>45282</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>ATYPICAL SQUAMOUS CELLS, CANNOT EXCLUDE HSIL (ASC-H)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Adequate</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1183,7 +1179,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>ASC-H</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1199,30 +1195,30 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PT00109</t>
+          <t>PT00100</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CYT-87304</t>
+          <t>CYT-58368</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>45567</v>
+        <v>45522</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>LSIL</t>
+          <t>HSIL. Features consistent with CIN 2-3. Colposcopy recommended.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Adequate</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>LBC</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1232,12 +1228,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>LSIL</t>
+          <t>HSIL</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1253,25 +1249,25 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PT00118</t>
+          <t>PT00125</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CYT-52372</t>
+          <t>CYT-17104</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>45185</v>
+        <v>45350</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>HIGH GRADE SQUAMOUS INTRAEPITHELIAL LESION (HSIL)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1291,7 +1287,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>HSIL</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1307,25 +1303,25 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PT00122</t>
+          <t>PT00127</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CYT-39451</t>
+          <t>CYT-92578</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>45022</v>
+        <v>44956</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Atypical glandular cells favor neoplasia</t>
+          <t>AGC-NEO. Endocervical adenocarcinoma in situ cannot be excluded.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactory for evaluation</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1335,7 +1331,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Dr. Lee</t>
+          <t>Dr. Patel</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1361,20 +1357,20 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PT00129</t>
+          <t>PT00142</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CYT-95461</t>
+          <t>CYT-13794</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>45606</v>
+        <v>45233</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Malignant cells present</t>
+          <t>Atypical squamous cells, undetermined significance. Reflex HPV testing recommended.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1384,66 +1380,62 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>Conventional</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Patel</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Clinic A</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>MALIGNANT</t>
-        </is>
-      </c>
+          <t>Outpatient</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PT00134</t>
+          <t>PT00144</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CYT-93066</t>
+          <t>CYT-89887</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>45027</v>
+        <v>45007</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Negative cytology</t>
+          <t>HSIL - SEE COMMENT. Correlate with clinical findings.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Adequate</t>
+          <t>Satisfactory for evaluation</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>LBC</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Dr. Patel</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1453,7 +1445,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>NILM</t>
+          <t>HSIL</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1469,25 +1461,25 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PT00139</t>
+          <t>PT00145</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CYT-30706</t>
+          <t>CYT-70443</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>45486</v>
+        <v>45164</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>AGC-NEO</t>
+          <t>ATYPICAL SQUAMOUS CELLS OF UNDETERMINED SIGNIFICANCE (ASC-US)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Adequate</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1497,17 +1489,17 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Dr. Lee</t>
+          <t>Dr. Smith</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Clinic A</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>AGC-NEO</t>
+          <t>ASC-US</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1523,30 +1515,30 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PT00145</t>
+          <t>PT00150</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CYT-52823</t>
+          <t>CYT-16428</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>45229</v>
+        <v>45629</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Atypical glandular cells</t>
+          <t>ATYPICAL GLANDULAR CELLS (AGC), NOT OTHERWISE SPECIFIED</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation</t>
+          <t>Adequate</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>Conventional</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">

</xml_diff>

<commit_message>
professional PDF report - LLM insights connected - encoding fixes - AI clinical commentary working
</commit_message>
<xml_diff>
--- a/data/output-data/unmatched_cases.xlsx
+++ b/data/output-data/unmatched_cases.xlsx
@@ -497,20 +497,20 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PT00001</t>
+          <t>PT00014</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CYT-24592</t>
+          <t>CYT-42325</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>45581</v>
+        <v>45069</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ATYPICAL GLANDULAR CELLS (AGC), NOT OTHERWISE SPECIFIED</t>
+          <t>OTHER (EMC45)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -520,22 +520,22 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>LBC</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Dr. Jones</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>OTHER (EMC45)</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -551,20 +551,20 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PT00008</t>
+          <t>PT00022</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CYT-19116</t>
+          <t>CYT-73699</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>45648</v>
+        <v>45014</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>ATYPICAL SQUAMOUS CELLS, CANNOT EXCLUDE HSIL (ASC-H)</t>
+          <t>Adenocarcinoma in situ</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -574,22 +574,22 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Conventional</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Dr. Smith</t>
+          <t>Dr. Lee</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Clinic A</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>ASC-H</t>
+          <t>AIS</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -605,20 +605,20 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PT00017</t>
+          <t>PT00037</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CYT-71348</t>
+          <t>CYT-79615</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>45537</v>
+        <v>45441</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ATYPICAL SQUAMOUS CELLS OF UNDETERMINED SIGNIFICANCE (ASC-US)</t>
+          <t>Neg</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -628,22 +628,22 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Smith</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Clinic A</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>ASC-US</t>
+          <t>NILM</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -659,35 +659,35 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PT00037</t>
+          <t>PT00041</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CYT-96752</t>
+          <t>CYT-11220</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>45496</v>
+        <v>45001</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>lsil</t>
+          <t>Endometrial cells</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation</t>
+          <t>Satisfactory</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Dr. Patel</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>LSIL</t>
+          <t>AGC-EMC</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -713,35 +713,35 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PT00041</t>
+          <t>PT00049</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CYT-85880</t>
+          <t>CYT-50404</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>45179</v>
+        <v>44969</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation. Negative for intraepithelial lesion or malignancy (NILM).</t>
+          <t>NILLM</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>LBC</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Jones</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -767,45 +767,45 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PT00055</t>
+          <t>PT00056</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CYT-53540</t>
+          <t>CYT-51114</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>45110</v>
+        <v>45280</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>AGC-NEO. Endocervical adenocarcinoma in situ cannot be excluded.</t>
+          <t>Carcinoma</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation</t>
+          <t>Satisfactory</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Conventional</t>
+          <t>LBC</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Dr. Jones</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Clinic A</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>AGC-NEO</t>
+          <t>MALIGNANT</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -821,95 +821,99 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PT00063</t>
+          <t>PT00062</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CYT-97410</t>
+          <t>CYT-38010</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>45243</v>
+        <v>45618</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Atypical squamous cells, undetermined significance. Reflex HPV testing recommended.</t>
+          <t>MALIGNANT</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Adequate</t>
+          <t>Satisfactory for evaluation</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Conventional</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Patel</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Main Lab</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
+          <t>Clinic A</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>MALIGNANT</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PT00067</t>
+          <t>PT00064</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CYT-97012</t>
+          <t>CYT-29313</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>45454</v>
+        <v>45130</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>HSIL - SEE COMMENT. Correlate with clinical findings.</t>
+          <t>NILLM</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Satisfactory for evaluation</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>LBC</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Dr. Jones</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Clinic A</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>HSIL</t>
+          <t>NILM</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -925,20 +929,20 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PT00071</t>
+          <t>PT00065</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CYT-77889</t>
+          <t>CYT-64321</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>45107</v>
+        <v>45393</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation. Negative for intraepithelial lesion or malignancy (NILM).</t>
+          <t>Endometrial cells</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -948,7 +952,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>LBC</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -958,12 +962,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>NILM</t>
+          <t>AGC-EMC</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -979,25 +983,25 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PT00078</t>
+          <t>PT00068</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CYT-86556</t>
+          <t>CYT-97500</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>45325</v>
+        <v>45402</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>NEGATIVE FOR INTRAEPITHELIAL LESION OR MALIGNANCY</t>
+          <t>OTHER (EMC45)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Adequate</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1007,17 +1011,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Dr. Smith</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Clinic A</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>NILM</t>
+          <t>OTHER (EMC45)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1033,45 +1037,45 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PT00085</t>
+          <t>PT00090</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CYT-95426</t>
+          <t>CYT-84691</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>44997</v>
+        <v>45402</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Atypical glandular cells, favor neoplasia. Further evaluation recommended.</t>
+          <t>ASC H</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Dr. Jones</t>
+          <t>Dr. Lee</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>AGC-NEO</t>
+          <t>ASC-H</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1087,20 +1091,20 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PT00089</t>
+          <t>PT00101</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CYT-92213</t>
+          <t>CYT-71524</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>45533</v>
+        <v>45218</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Negative. No significant atypia identified.</t>
+          <t>AGC-NEO</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1110,22 +1114,22 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Smith</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>NILM</t>
+          <t>AGC-NEO</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1141,25 +1145,25 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PT00090</t>
+          <t>PT00102</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CYT-79827</t>
+          <t>CYT-24953</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>45282</v>
+        <v>45416</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>ATYPICAL SQUAMOUS CELLS, CANNOT EXCLUDE HSIL (ASC-H)</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Adequate</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1179,7 +1183,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>ASC-H</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1195,30 +1199,30 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PT00100</t>
+          <t>PT00109</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CYT-58368</t>
+          <t>CYT-87304</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>45522</v>
+        <v>45567</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>HSIL. Features consistent with CIN 2-3. Colposcopy recommended.</t>
+          <t>LSIL</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Adequate</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>LBC</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1228,12 +1232,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>HSIL</t>
+          <t>LSIL</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1249,25 +1253,25 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PT00125</t>
+          <t>PT00118</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CYT-17104</t>
+          <t>CYT-52372</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>45350</v>
+        <v>45185</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>HIGH GRADE SQUAMOUS INTRAEPITHELIAL LESION (HSIL)</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Satisfactory</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1287,7 +1291,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>HSIL</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1303,25 +1307,25 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PT00127</t>
+          <t>PT00122</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CYT-92578</t>
+          <t>CYT-39451</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>44956</v>
+        <v>45022</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>AGC-NEO. Endocervical adenocarcinoma in situ cannot be excluded.</t>
+          <t>Atypical glandular cells favor neoplasia</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation</t>
+          <t>Satisfactory</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1331,7 +1335,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Dr. Patel</t>
+          <t>Dr. Lee</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1357,20 +1361,20 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PT00142</t>
+          <t>PT00129</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CYT-13794</t>
+          <t>CYT-95461</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>45233</v>
+        <v>45606</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Atypical squamous cells, undetermined significance. Reflex HPV testing recommended.</t>
+          <t>Malignant cells present</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1380,62 +1384,66 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Conventional</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Dr. Patel</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Outpatient</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr"/>
+          <t>Clinic A</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>MALIGNANT</t>
+        </is>
+      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PT00144</t>
+          <t>PT00134</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CYT-89887</t>
+          <t>CYT-93066</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>45007</v>
+        <v>45027</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>HSIL - SEE COMMENT. Correlate with clinical findings.</t>
+          <t>Negative cytology</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation</t>
+          <t>Adequate</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>LBC</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Patel</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1445,7 +1453,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>HSIL</t>
+          <t>NILM</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1461,25 +1469,25 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PT00145</t>
+          <t>PT00139</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CYT-70443</t>
+          <t>CYT-30706</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>45164</v>
+        <v>45486</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>ATYPICAL SQUAMOUS CELLS OF UNDETERMINED SIGNIFICANCE (ASC-US)</t>
+          <t>AGC-NEO</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Adequate</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1489,17 +1497,17 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Dr. Smith</t>
+          <t>Dr. Lee</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Clinic A</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>ASC-US</t>
+          <t>AGC-NEO</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1515,30 +1523,30 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PT00150</t>
+          <t>PT00145</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CYT-16428</t>
+          <t>CYT-52823</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>45629</v>
+        <v>45229</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>ATYPICAL GLANDULAR CELLS (AGC), NOT OTHERWISE SPECIFIED</t>
+          <t>Atypical glandular cells</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Adequate</t>
+          <t>Satisfactory for evaluation</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Conventional</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">

</xml_diff>

<commit_message>
add demo mode for Streamlit Cloud deployment - wrap Ollama calls
</commit_message>
<xml_diff>
--- a/data/output-data/unmatched_cases.xlsx
+++ b/data/output-data/unmatched_cases.xlsx
@@ -497,20 +497,20 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PT00014</t>
+          <t>PT00001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CYT-42325</t>
+          <t>CYT-24592</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>45069</v>
+        <v>45581</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>OTHER (EMC45)</t>
+          <t>ATYPICAL GLANDULAR CELLS (AGC), NOT OTHERWISE SPECIFIED</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -520,22 +520,22 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>LBC</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Jones</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>OTHER (EMC45)</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -551,20 +551,20 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PT00022</t>
+          <t>PT00008</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CYT-73699</t>
+          <t>CYT-19116</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>45014</v>
+        <v>45648</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Adenocarcinoma in situ</t>
+          <t>ATYPICAL SQUAMOUS CELLS, CANNOT EXCLUDE HSIL (ASC-H)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -574,22 +574,22 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>Conventional</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Dr. Lee</t>
+          <t>Dr. Smith</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Clinic A</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>AIS</t>
+          <t>ASC-H</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -605,20 +605,20 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PT00037</t>
+          <t>PT00017</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CYT-79615</t>
+          <t>CYT-71348</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>45441</v>
+        <v>45537</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Neg</t>
+          <t>ATYPICAL SQUAMOUS CELLS OF UNDETERMINED SIGNIFICANCE (ASC-US)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -628,22 +628,22 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Dr. Smith</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Clinic A</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>NILM</t>
+          <t>ASC-US</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -659,35 +659,35 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PT00041</t>
+          <t>PT00037</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CYT-11220</t>
+          <t>CYT-96752</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>45001</v>
+        <v>45496</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Endometrial cells</t>
+          <t>lsil</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactory for evaluation</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Patel</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>AGC-EMC</t>
+          <t>LSIL</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -713,35 +713,35 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PT00049</t>
+          <t>PT00041</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CYT-50404</t>
+          <t>CYT-85880</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>44969</v>
+        <v>45179</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>NILLM</t>
+          <t>Satisfactory for evaluation. Negative for intraepithelial lesion or malignancy (NILM).</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Satisfactory</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>LBC</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Dr. Jones</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -767,45 +767,45 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PT00056</t>
+          <t>PT00055</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CYT-51114</t>
+          <t>CYT-53540</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>45280</v>
+        <v>45110</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Carcinoma</t>
+          <t>AGC-NEO. Endocervical adenocarcinoma in situ cannot be excluded.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactory for evaluation</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>LBC</t>
+          <t>Conventional</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Jones</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Clinic A</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>MALIGNANT</t>
+          <t>AGC-NEO</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -821,99 +821,95 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PT00062</t>
+          <t>PT00063</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CYT-38010</t>
+          <t>CYT-97410</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>45618</v>
+        <v>45243</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MALIGNANT</t>
+          <t>Atypical squamous cells, undetermined significance. Reflex HPV testing recommended.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation</t>
+          <t>Adequate</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>Conventional</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Dr. Patel</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Clinic A</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>MALIGNANT</t>
-        </is>
-      </c>
+          <t>Main Lab</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PT00064</t>
+          <t>PT00067</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CYT-29313</t>
+          <t>CYT-97012</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>45130</v>
+        <v>45454</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>NILLM</t>
+          <t>HSIL - SEE COMMENT. Correlate with clinical findings.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>LBC</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Jones</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Clinic A</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>NILM</t>
+          <t>HSIL</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -929,20 +925,20 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PT00065</t>
+          <t>PT00071</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CYT-64321</t>
+          <t>CYT-77889</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>45393</v>
+        <v>45107</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Endometrial cells</t>
+          <t>Satisfactory for evaluation. Negative for intraepithelial lesion or malignancy (NILM).</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -952,7 +948,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>LBC</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -962,12 +958,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>AGC-EMC</t>
+          <t>NILM</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -983,25 +979,25 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PT00068</t>
+          <t>PT00078</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CYT-97500</t>
+          <t>CYT-86556</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>45402</v>
+        <v>45325</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>OTHER (EMC45)</t>
+          <t>NEGATIVE FOR INTRAEPITHELIAL LESION OR MALIGNANCY</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Adequate</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1011,17 +1007,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Smith</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Clinic A</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>OTHER (EMC45)</t>
+          <t>NILM</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1037,45 +1033,45 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PT00090</t>
+          <t>PT00085</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CYT-84691</t>
+          <t>CYT-95426</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>45402</v>
+        <v>44997</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ASC H</t>
+          <t>Atypical glandular cells, favor neoplasia. Further evaluation recommended.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Satisfactory</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>SurePath</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Dr. Lee</t>
+          <t>Dr. Jones</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>ASC-H</t>
+          <t>AGC-NEO</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1091,20 +1087,20 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PT00101</t>
+          <t>PT00089</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CYT-71524</t>
+          <t>CYT-92213</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>45218</v>
+        <v>45533</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>AGC-NEO</t>
+          <t>Negative. No significant atypia identified.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1114,22 +1110,22 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>ThinPrep</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Dr. Smith</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Outpatient</t>
+          <t>Main Lab</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>AGC-NEO</t>
+          <t>NILM</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1145,25 +1141,25 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PT00102</t>
+          <t>PT00090</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CYT-24953</t>
+          <t>CYT-79827</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>45416</v>
+        <v>45282</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>ATYPICAL SQUAMOUS CELLS, CANNOT EXCLUDE HSIL (ASC-H)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Adequate</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1183,7 +1179,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>ASC-H</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1199,30 +1195,30 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PT00109</t>
+          <t>PT00100</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CYT-87304</t>
+          <t>CYT-58368</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>45567</v>
+        <v>45522</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>LSIL</t>
+          <t>HSIL. Features consistent with CIN 2-3. Colposcopy recommended.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Adequate</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>ThinPrep</t>
+          <t>LBC</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1232,12 +1228,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Main Lab</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>LSIL</t>
+          <t>HSIL</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1253,25 +1249,25 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PT00118</t>
+          <t>PT00125</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CYT-52372</t>
+          <t>CYT-17104</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>45185</v>
+        <v>45350</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>HIGH GRADE SQUAMOUS INTRAEPITHELIAL LESION (HSIL)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Unsatisfactory</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1291,7 +1287,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>HSIL</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1307,25 +1303,25 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PT00122</t>
+          <t>PT00127</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CYT-39451</t>
+          <t>CYT-92578</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>45022</v>
+        <v>44956</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Atypical glandular cells favor neoplasia</t>
+          <t>AGC-NEO. Endocervical adenocarcinoma in situ cannot be excluded.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactory for evaluation</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1335,7 +1331,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Dr. Lee</t>
+          <t>Dr. Patel</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1361,20 +1357,20 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PT00129</t>
+          <t>PT00142</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CYT-95461</t>
+          <t>CYT-13794</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>45606</v>
+        <v>45233</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Malignant cells present</t>
+          <t>Atypical squamous cells, undetermined significance. Reflex HPV testing recommended.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1384,66 +1380,62 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>Conventional</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Dr. Kim</t>
+          <t>Dr. Patel</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Clinic A</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>MALIGNANT</t>
-        </is>
-      </c>
+          <t>Outpatient</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PT00134</t>
+          <t>PT00144</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CYT-93066</t>
+          <t>CYT-89887</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>45027</v>
+        <v>45007</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Negative cytology</t>
+          <t>HSIL - SEE COMMENT. Correlate with clinical findings.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Adequate</t>
+          <t>Satisfactory for evaluation</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>LBC</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Dr. Patel</t>
+          <t>Dr. Kim</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1453,7 +1445,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>NILM</t>
+          <t>HSIL</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1469,25 +1461,25 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PT00139</t>
+          <t>PT00145</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CYT-30706</t>
+          <t>CYT-70443</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>45486</v>
+        <v>45164</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>AGC-NEO</t>
+          <t>ATYPICAL SQUAMOUS CELLS OF UNDETERMINED SIGNIFICANCE (ASC-US)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Unsatisfactory</t>
+          <t>Adequate</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1497,17 +1489,17 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Dr. Lee</t>
+          <t>Dr. Smith</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Clinic A</t>
+          <t>Outpatient</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>AGC-NEO</t>
+          <t>ASC-US</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1523,30 +1515,30 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PT00145</t>
+          <t>PT00150</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CYT-52823</t>
+          <t>CYT-16428</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>45229</v>
+        <v>45629</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Atypical glandular cells</t>
+          <t>ATYPICAL GLANDULAR CELLS (AGC), NOT OTHERWISE SPECIFIED</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Satisfactory for evaluation</t>
+          <t>Adequate</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>SurePath</t>
+          <t>Conventional</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">

</xml_diff>